<commit_message>
MS data used if LC data is blank and run numbers added
</commit_message>
<xml_diff>
--- a/output/worklist_conditions_project_26.xlsx
+++ b/output/worklist_conditions_project_26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DD0C7DD-BA49-E548-AF39-AB081EBF1E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FC4D02-44D1-1D44-AE9D-A276B7E4FC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="99">
   <si>
     <t>Number:</t>
   </si>
@@ -309,18 +309,6 @@
     <t>msmethodfilename</t>
   </si>
   <si>
-    <t>lcdatapath</t>
-  </si>
-  <si>
-    <t>lcmethodpath</t>
-  </si>
-  <si>
-    <t>lcmethod</t>
-  </si>
-  <si>
-    <t>lcmethodfilename</t>
-  </si>
-  <si>
     <t>Y</t>
   </si>
   <si>
@@ -342,7 +330,7 @@
     <t>System configuration:</t>
   </si>
   <si>
-    <t>Thermo</t>
+    <t>Bruker</t>
   </si>
 </sst>
 </file>
@@ -1535,7 +1523,7 @@
     </row>
     <row r="9" spans="1:48" x14ac:dyDescent="0.2">
       <c r="B9" s="31" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D9" t="s">
         <v>52</v>
@@ -2666,7 +2654,7 @@
     </row>
     <row r="27" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B27" s="31" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D27" t="s">
         <v>52</v>
@@ -3436,7 +3424,7 @@
     </row>
     <row r="45" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="31" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D45" t="s">
         <v>52</v>
@@ -3946,7 +3934,7 @@
         <v>38</v>
       </c>
       <c r="D59" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -4028,7 +4016,7 @@
     </row>
     <row r="60" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A60" s="41" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B60" s="13"/>
       <c r="D60" t="s">
@@ -4122,7 +4110,7 @@
     </row>
     <row r="63" spans="1:40" x14ac:dyDescent="0.2">
       <c r="B63" s="31" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D63" t="s">
         <v>52</v>
@@ -4629,7 +4617,7 @@
         <v>12</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>13</v>
@@ -4641,7 +4629,7 @@
         <v>15</v>
       </c>
       <c r="R1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
@@ -4668,18 +4656,10 @@
       <c r="G2" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H2" s="8"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="8"/>
       <c r="L2" s="29" t="str">
         <f>IF(LEN(User!AG2)=0,"",User!AG2)</f>
         <v/>
@@ -4720,18 +4700,10 @@
       <c r="G3" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H3" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K3" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H3" s="8"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="8"/>
       <c r="L3" s="29" t="str">
         <f>IF(LEN(User!AG3)=0,"",User!AG3)</f>
         <v/>
@@ -4769,18 +4741,10 @@
       <c r="G4" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H4" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H4" s="8"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="8"/>
       <c r="L4" s="29" t="str">
         <f>IF(LEN(User!AG4)=0,"",User!AG4)</f>
         <v/>
@@ -4817,18 +4781,10 @@
       <c r="G5" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H5" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H5" s="8"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="8"/>
       <c r="L5" s="29" t="str">
         <f>IF(LEN(User!AG5)=0,"",User!AG5)</f>
         <v/>
@@ -4871,18 +4827,10 @@
       <c r="G6" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H6" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H6" s="8"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="8"/>
       <c r="L6" s="29" t="str">
         <f>IF(LEN(User!AG6)=0,"",User!AG6)</f>
         <v/>
@@ -4923,18 +4871,10 @@
       <c r="G7" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H7" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H7" s="8"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="8"/>
       <c r="L7" s="29" t="str">
         <f>IF(LEN(User!AG7)=0,"",User!AG7)</f>
         <v/>
@@ -4971,18 +4911,10 @@
       <c r="G8" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H8" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H8" s="8"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="8"/>
       <c r="L8" s="29" t="str">
         <f>IF(LEN(User!AG8)=0,"",User!AG8)</f>
         <v/>
@@ -5025,18 +4957,10 @@
       <c r="G9" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H9" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H9" s="8"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="8"/>
       <c r="L9" s="29" t="str">
         <f>IF(LEN(User!AG9)=0,"",User!AG9)</f>
         <v/>
@@ -5085,18 +5009,10 @@
       <c r="G10" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H10" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H10" s="8"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="8"/>
       <c r="L10" s="29" t="str">
         <f>IF(LEN(User!AG10)=0,"",User!AG10)</f>
         <v/>
@@ -5141,18 +5057,10 @@
       <c r="G11" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H11" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H11" s="8"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="8"/>
       <c r="L11" s="29" t="str">
         <f>IF(LEN(User!AG11)=0,"",User!AG11)</f>
         <v/>
@@ -5187,18 +5095,10 @@
       <c r="G12" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H12" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K12" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H12" s="8"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="8"/>
       <c r="L12" s="29" t="str">
         <f>IF(LEN(User!AG12)=0,"",User!AG12)</f>
         <v/>
@@ -5239,18 +5139,10 @@
       <c r="G13" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H13" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H13" s="8"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="8"/>
       <c r="L13" s="29" t="str">
         <f>IF(LEN(User!AG13)=0,"",User!AG13)</f>
         <v/>
@@ -5291,18 +5183,10 @@
       <c r="G14" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="H14" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>94</v>
-      </c>
+      <c r="H14" s="8"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="8"/>
       <c r="L14" s="29" t="str">
         <f>IF(LEN(User!AG14)=0,"",User!AG14)</f>
         <v/>
@@ -5319,10 +5203,10 @@
         <v>1</v>
       </c>
       <c r="R14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="S14" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="S14" s="6" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
@@ -5355,7 +5239,7 @@
       <c r="P15" s="11"/>
       <c r="Q15" s="11"/>
       <c r="R15" s="43" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="S15" s="44"/>
     </row>

</xml_diff>

<commit_message>
solvent vial multiplier added
</commit_message>
<xml_diff>
--- a/output/worklist_conditions_project_26.xlsx
+++ b/output/worklist_conditions_project_26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7C6407-2CD6-E640-876C-CA8BB583F4E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F260B3-C953-FE49-B6C5-EF2ED76BF8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2063,6 +2063,9 @@
       <c r="AF14" s="7" t="s">
         <v>80</v>
       </c>
+      <c r="AG14" s="29">
+        <v>200</v>
+      </c>
       <c r="AM14" s="10"/>
       <c r="AN14" s="10"/>
       <c r="AO14" s="30"/>
@@ -2102,9 +2105,7 @@
       </c>
       <c r="AE15" s="8"/>
       <c r="AF15" s="7"/>
-      <c r="AG15" s="29">
-        <v>200</v>
-      </c>
+      <c r="AG15" s="29"/>
       <c r="AM15" s="10"/>
       <c r="AN15" s="10"/>
       <c r="AO15" s="30"/>
@@ -5189,7 +5190,7 @@
       <c r="J14" s="7"/>
       <c r="K14" s="8"/>
       <c r="L14" s="29">
-        <f>IF(LEN(User!AG15)=0,"",User!AG15)</f>
+        <f>IF(LEN(User!AG14)=0,"",User!AG14)</f>
         <v>200</v>
       </c>
       <c r="M14" s="12"/>
@@ -5230,9 +5231,9 @@
       <c r="I15" s="7"/>
       <c r="J15" s="7"/>
       <c r="K15" s="8"/>
-      <c r="L15" s="29" t="e">
-        <f>IF(LEN(User!#REF!)=0,"",User!#REF!)</f>
-        <v>#REF!</v>
+      <c r="L15" s="29" t="str">
+        <f>IF(LEN(User!AG15)=0,"",User!AG15)</f>
+        <v/>
       </c>
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>

</xml_diff>

<commit_message>
added random seed implementation
</commit_message>
<xml_diff>
--- a/output/worklist_conditions_project_26.xlsx
+++ b/output/worklist_conditions_project_26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06F260B3-C953-FE49-B6C5-EF2ED76BF8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280D7931-FB15-AB45-8C72-274B466A1F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="101">
   <si>
     <t>Number:</t>
   </si>
@@ -331,13 +331,19 @@
   </si>
   <si>
     <t>Bruker</t>
+  </si>
+  <si>
+    <t>Random seed:</t>
+  </si>
+  <si>
+    <t>Optional setting of random seed for consistent randomization</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -363,6 +369,11 @@
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow (Cuerpo)"/>
     </font>
   </fonts>
   <fills count="5">
@@ -572,7 +583,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
@@ -661,18 +672,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -689,6 +688,24 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1121,10 +1138,10 @@
       <c r="AM3" s="10"/>
       <c r="AN3" s="10"/>
       <c r="AO3" s="30"/>
-      <c r="AU3" s="51" t="s">
+      <c r="AU3" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="AV3" s="50"/>
+      <c r="AV3" s="46"/>
     </row>
     <row r="4" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
@@ -1168,15 +1185,15 @@
         <v>35</v>
       </c>
       <c r="AJ4" s="6"/>
-      <c r="AK4" s="49" t="s">
+      <c r="AK4" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="AL4" s="50"/>
+      <c r="AL4" s="46"/>
       <c r="AM4" s="10"/>
       <c r="AN4" s="10"/>
       <c r="AO4" s="30"/>
-      <c r="AU4" s="50"/>
-      <c r="AV4" s="50"/>
+      <c r="AU4" s="46"/>
+      <c r="AV4" s="46"/>
     </row>
     <row r="5" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
@@ -1276,15 +1293,15 @@
       <c r="AJ5" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="AK5" s="49" t="s">
+      <c r="AK5" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="AL5" s="50"/>
+      <c r="AL5" s="46"/>
       <c r="AM5" s="10"/>
       <c r="AN5" s="10"/>
       <c r="AO5" s="30"/>
-      <c r="AU5" s="50"/>
-      <c r="AV5" s="50"/>
+      <c r="AU5" s="46"/>
+      <c r="AV5" s="46"/>
     </row>
     <row r="6" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A6" s="41" t="s">
@@ -1332,8 +1349,8 @@
       <c r="AM6" s="10"/>
       <c r="AN6" s="10"/>
       <c r="AO6" s="30"/>
-      <c r="AU6" s="50"/>
-      <c r="AV6" s="50"/>
+      <c r="AU6" s="46"/>
+      <c r="AV6" s="46"/>
     </row>
     <row r="7" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D7" t="s">
@@ -1420,8 +1437,8 @@
       <c r="AM7" s="10"/>
       <c r="AN7" s="10"/>
       <c r="AO7" s="30"/>
-      <c r="AU7" s="50"/>
-      <c r="AV7" s="50"/>
+      <c r="AU7" s="46"/>
+      <c r="AV7" s="46"/>
     </row>
     <row r="8" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D8" t="s">
@@ -1511,15 +1528,15 @@
       <c r="AJ8" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="AK8" s="49" t="s">
+      <c r="AK8" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="AL8" s="50"/>
+      <c r="AL8" s="46"/>
       <c r="AM8" s="10"/>
       <c r="AN8" s="10"/>
       <c r="AO8" s="30"/>
-      <c r="AU8" s="50"/>
-      <c r="AV8" s="50"/>
+      <c r="AU8" s="46"/>
+      <c r="AV8" s="46"/>
     </row>
     <row r="9" spans="1:48" x14ac:dyDescent="0.2">
       <c r="B9" s="31" t="s">
@@ -1610,13 +1627,13 @@
         <v>53</v>
       </c>
       <c r="AJ9" s="6"/>
-      <c r="AK9" s="52"/>
-      <c r="AL9" s="50"/>
+      <c r="AK9" s="48"/>
+      <c r="AL9" s="46"/>
       <c r="AM9" s="10"/>
       <c r="AN9" s="10"/>
       <c r="AO9" s="30"/>
-      <c r="AU9" s="50"/>
-      <c r="AV9" s="50"/>
+      <c r="AU9" s="46"/>
+      <c r="AV9" s="46"/>
     </row>
     <row r="10" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A10">
@@ -1706,19 +1723,19 @@
         <v>71</v>
       </c>
       <c r="AG10" s="29"/>
-      <c r="AI10" s="53" t="s">
+      <c r="AI10" s="49" t="s">
         <v>55</v>
       </c>
-      <c r="AJ10" s="55" t="s">
+      <c r="AJ10" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="AK10" s="52"/>
-      <c r="AL10" s="50"/>
+      <c r="AK10" s="48"/>
+      <c r="AL10" s="46"/>
       <c r="AM10" s="10"/>
       <c r="AN10" s="10"/>
       <c r="AO10" s="30"/>
-      <c r="AU10" s="50"/>
-      <c r="AV10" s="50"/>
+      <c r="AU10" s="46"/>
+      <c r="AV10" s="46"/>
     </row>
     <row r="11" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A11">
@@ -1806,15 +1823,15 @@
         <v>75</v>
       </c>
       <c r="AG11" s="29"/>
-      <c r="AI11" s="54"/>
-      <c r="AJ11" s="56"/>
+      <c r="AI11" s="50"/>
+      <c r="AJ11" s="52"/>
       <c r="AK11" s="32"/>
       <c r="AL11" s="32"/>
       <c r="AM11" s="10"/>
       <c r="AN11" s="10"/>
       <c r="AO11" s="30"/>
-      <c r="AU11" s="50"/>
-      <c r="AV11" s="50"/>
+      <c r="AU11" s="46"/>
+      <c r="AV11" s="46"/>
     </row>
     <row r="12" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A12">
@@ -1899,8 +1916,8 @@
       <c r="AM12" s="10"/>
       <c r="AN12" s="10"/>
       <c r="AO12" s="30"/>
-      <c r="AU12" s="50"/>
-      <c r="AV12" s="50"/>
+      <c r="AU12" s="46"/>
+      <c r="AV12" s="46"/>
     </row>
     <row r="13" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A13">
@@ -1985,8 +2002,8 @@
       <c r="AM13" s="10"/>
       <c r="AN13" s="10"/>
       <c r="AO13" s="30"/>
-      <c r="AU13" s="50"/>
-      <c r="AV13" s="50"/>
+      <c r="AU13" s="46"/>
+      <c r="AV13" s="46"/>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A14">
@@ -2063,14 +2080,12 @@
       <c r="AF14" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="AG14" s="29">
-        <v>200</v>
-      </c>
+      <c r="AG14" s="29"/>
       <c r="AM14" s="10"/>
       <c r="AN14" s="10"/>
       <c r="AO14" s="30"/>
-      <c r="AU14" s="50"/>
-      <c r="AV14" s="50"/>
+      <c r="AU14" s="46"/>
+      <c r="AV14" s="46"/>
     </row>
     <row r="15" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D15" t="s">
@@ -4844,10 +4859,10 @@
       <c r="O6" s="12"/>
       <c r="P6" s="11"/>
       <c r="Q6" s="11"/>
-      <c r="R6" s="47" t="s">
+      <c r="R6" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="S6" s="48"/>
+      <c r="S6" s="56"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="12">
@@ -5030,10 +5045,10 @@
       <c r="Q10" s="11">
         <v>1</v>
       </c>
-      <c r="R10" s="45" t="s">
+      <c r="R10" s="53" t="s">
         <v>22</v>
       </c>
-      <c r="S10" s="46"/>
+      <c r="S10" s="54"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="12">
@@ -5156,10 +5171,10 @@
       <c r="O13" s="12"/>
       <c r="P13" s="11"/>
       <c r="Q13" s="11"/>
-      <c r="R13" s="45" t="s">
+      <c r="R13" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="S13" s="46"/>
+      <c r="S13" s="54"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="12">
@@ -5189,9 +5204,9 @@
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
       <c r="K14" s="8"/>
-      <c r="L14" s="29">
+      <c r="L14" s="29" t="str">
         <f>IF(LEN(User!AG14)=0,"",User!AG14)</f>
-        <v>200</v>
+        <v/>
       </c>
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
@@ -5274,8 +5289,14 @@
       <c r="O16" s="12"/>
       <c r="P16" s="11"/>
       <c r="Q16" s="11"/>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R16" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="S16" s="6">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="12">
         <v>16</v>
       </c>
@@ -5304,8 +5325,12 @@
       <c r="O17" s="12"/>
       <c r="P17" s="11"/>
       <c r="Q17" s="11"/>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R17" s="58" t="s">
+        <v>100</v>
+      </c>
+      <c r="S17" s="57"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="12">
         <v>17</v>
       </c>
@@ -5335,7 +5360,7 @@
       <c r="P18" s="11"/>
       <c r="Q18" s="11"/>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="12">
         <v>18</v>
       </c>
@@ -5365,7 +5390,7 @@
       <c r="P19" s="11"/>
       <c r="Q19" s="11"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="12">
         <v>19</v>
       </c>
@@ -5395,7 +5420,7 @@
       <c r="P20" s="11"/>
       <c r="Q20" s="11"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="12">
         <v>20</v>
       </c>
@@ -5425,7 +5450,7 @@
       <c r="P21" s="11"/>
       <c r="Q21" s="11"/>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" s="12">
         <v>21</v>
       </c>
@@ -5455,7 +5480,7 @@
       <c r="P22" s="11"/>
       <c r="Q22" s="11"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A23" s="12">
         <v>22</v>
       </c>
@@ -5485,7 +5510,7 @@
       <c r="P23" s="11"/>
       <c r="Q23" s="11"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" s="12">
         <v>23</v>
       </c>
@@ -5514,7 +5539,7 @@
       <c r="P24" s="11"/>
       <c r="Q24" s="11"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" s="12">
         <v>24</v>
       </c>
@@ -5544,7 +5569,7 @@
       <c r="P25" s="11"/>
       <c r="Q25" s="11"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" s="12">
         <v>25</v>
       </c>
@@ -5574,7 +5599,7 @@
       <c r="P26" s="11"/>
       <c r="Q26" s="11"/>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="12">
         <v>26</v>
       </c>
@@ -5604,7 +5629,7 @@
       <c r="P27" s="11"/>
       <c r="Q27" s="11"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" s="12">
         <v>27</v>
       </c>
@@ -5634,7 +5659,7 @@
       <c r="P28" s="11"/>
       <c r="Q28" s="11"/>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" s="12">
         <v>28</v>
       </c>
@@ -5664,7 +5689,7 @@
       <c r="P29" s="11"/>
       <c r="Q29" s="11"/>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" s="12">
         <v>29</v>
       </c>
@@ -5694,7 +5719,7 @@
       <c r="P30" s="11"/>
       <c r="Q30" s="11"/>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" s="12">
         <v>30</v>
       </c>
@@ -5724,7 +5749,7 @@
       <c r="P31" s="11"/>
       <c r="Q31" s="11"/>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" s="12">
         <v>31</v>
       </c>
@@ -6320,12 +6345,13 @@
       <c r="Q51" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="R13:S13"/>
     <mergeCell ref="R10:S10"/>
     <mergeCell ref="R6:S6"/>
+    <mergeCell ref="R17:S17"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:C51" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Condition,QC,Blank,TrueBlank,Lib,SystemValidation,WetQC"</formula1>
     </dataValidation>
@@ -6341,6 +6367,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S14" xr:uid="{DD0C5D8A-2183-E546-AA75-585BBC29853B}">
       <formula1>"(choose),Thermo,Bruker"</formula1>
     </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S16" xr:uid="{CC569B2F-CC74-6E41-8BBF-F55B73B7D6CB}">
+      <formula1>0</formula1>
+      <formula2>9999999999999990000</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
added example templates before and after
</commit_message>
<xml_diff>
--- a/output/worklist_conditions_project_26.xlsx
+++ b/output/worklist_conditions_project_26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280D7931-FB15-AB45-8C72-274B466A1F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE56D84-DD2D-AF49-8065-82516EE5F102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5292,9 +5292,7 @@
       <c r="R16" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="S16" s="6">
-        <v>42</v>
-      </c>
+      <c r="S16" s="6"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="12">

</xml_diff>

<commit_message>
added SDRF functionality and updated required fields
</commit_message>
<xml_diff>
--- a/output/worklist_conditions_project_26.xlsx
+++ b/output/worklist_conditions_project_26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE56D84-DD2D-AF49-8065-82516EE5F102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFFC109F-218A-5F4B-8F2D-2E36162500FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="99">
   <si>
     <t>Number:</t>
   </si>
@@ -279,18 +279,12 @@
     <t>qc2</t>
   </si>
   <si>
-    <t>R5</t>
-  </si>
-  <si>
     <t>1 column</t>
   </si>
   <si>
     <t>Before</t>
   </si>
   <si>
-    <t>UltiMate3000</t>
-  </si>
-  <si>
     <t>GW0409</t>
   </si>
   <si>
@@ -330,13 +324,13 @@
     <t>System configuration:</t>
   </si>
   <si>
-    <t>Bruker</t>
-  </si>
-  <si>
     <t>Random seed:</t>
   </si>
   <si>
     <t>Optional setting of random seed for consistent randomization</t>
+  </si>
+  <si>
+    <t>(choose)</t>
   </si>
 </sst>
 </file>
@@ -672,6 +666,24 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -688,24 +700,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1069,7 +1063,7 @@
         <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="AD1" s="5" t="s">
         <v>0</v>
@@ -1094,7 +1088,7 @@
         <v>27</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="AD2" s="12">
         <v>1</v>
@@ -1138,10 +1132,10 @@
       <c r="AM3" s="10"/>
       <c r="AN3" s="10"/>
       <c r="AO3" s="30"/>
-      <c r="AU3" s="47" t="s">
+      <c r="AU3" s="53" t="s">
         <v>33</v>
       </c>
-      <c r="AV3" s="46"/>
+      <c r="AV3" s="52"/>
     </row>
     <row r="4" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
@@ -1185,15 +1179,15 @@
         <v>35</v>
       </c>
       <c r="AJ4" s="6"/>
-      <c r="AK4" s="45" t="s">
+      <c r="AK4" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="AL4" s="46"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="10"/>
       <c r="AN4" s="10"/>
       <c r="AO4" s="30"/>
-      <c r="AU4" s="46"/>
-      <c r="AV4" s="46"/>
+      <c r="AU4" s="52"/>
+      <c r="AV4" s="52"/>
     </row>
     <row r="5" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
@@ -1290,18 +1284,16 @@
       <c r="AI5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AJ5" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="AK5" s="45" t="s">
+      <c r="AJ5" s="6"/>
+      <c r="AK5" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="AL5" s="46"/>
+      <c r="AL5" s="52"/>
       <c r="AM5" s="10"/>
       <c r="AN5" s="10"/>
       <c r="AO5" s="30"/>
-      <c r="AU5" s="46"/>
-      <c r="AV5" s="46"/>
+      <c r="AU5" s="52"/>
+      <c r="AV5" s="52"/>
     </row>
     <row r="6" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A6" s="41" t="s">
@@ -1349,8 +1341,8 @@
       <c r="AM6" s="10"/>
       <c r="AN6" s="10"/>
       <c r="AO6" s="30"/>
-      <c r="AU6" s="46"/>
-      <c r="AV6" s="46"/>
+      <c r="AU6" s="52"/>
+      <c r="AV6" s="52"/>
     </row>
     <row r="7" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D7" t="s">
@@ -1437,8 +1429,8 @@
       <c r="AM7" s="10"/>
       <c r="AN7" s="10"/>
       <c r="AO7" s="30"/>
-      <c r="AU7" s="46"/>
-      <c r="AV7" s="46"/>
+      <c r="AU7" s="52"/>
+      <c r="AV7" s="52"/>
     </row>
     <row r="8" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D8" t="s">
@@ -1528,19 +1520,19 @@
       <c r="AJ8" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="AK8" s="45" t="s">
+      <c r="AK8" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="AL8" s="46"/>
+      <c r="AL8" s="52"/>
       <c r="AM8" s="10"/>
       <c r="AN8" s="10"/>
       <c r="AO8" s="30"/>
-      <c r="AU8" s="46"/>
-      <c r="AV8" s="46"/>
+      <c r="AU8" s="52"/>
+      <c r="AV8" s="52"/>
     </row>
     <row r="9" spans="1:48" x14ac:dyDescent="0.2">
       <c r="B9" s="31" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D9" t="s">
         <v>52</v>
@@ -1627,13 +1619,13 @@
         <v>53</v>
       </c>
       <c r="AJ9" s="6"/>
-      <c r="AK9" s="48"/>
-      <c r="AL9" s="46"/>
+      <c r="AK9" s="54"/>
+      <c r="AL9" s="52"/>
       <c r="AM9" s="10"/>
       <c r="AN9" s="10"/>
       <c r="AO9" s="30"/>
-      <c r="AU9" s="46"/>
-      <c r="AV9" s="46"/>
+      <c r="AU9" s="52"/>
+      <c r="AV9" s="52"/>
     </row>
     <row r="10" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A10">
@@ -1723,19 +1715,19 @@
         <v>71</v>
       </c>
       <c r="AG10" s="29"/>
-      <c r="AI10" s="49" t="s">
+      <c r="AI10" s="55" t="s">
         <v>55</v>
       </c>
-      <c r="AJ10" s="51" t="s">
+      <c r="AJ10" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="AK10" s="48"/>
-      <c r="AL10" s="46"/>
+      <c r="AK10" s="54"/>
+      <c r="AL10" s="52"/>
       <c r="AM10" s="10"/>
       <c r="AN10" s="10"/>
       <c r="AO10" s="30"/>
-      <c r="AU10" s="46"/>
-      <c r="AV10" s="46"/>
+      <c r="AU10" s="52"/>
+      <c r="AV10" s="52"/>
     </row>
     <row r="11" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A11">
@@ -1823,15 +1815,15 @@
         <v>75</v>
       </c>
       <c r="AG11" s="29"/>
-      <c r="AI11" s="50"/>
-      <c r="AJ11" s="52"/>
+      <c r="AI11" s="56"/>
+      <c r="AJ11" s="58"/>
       <c r="AK11" s="32"/>
       <c r="AL11" s="32"/>
       <c r="AM11" s="10"/>
       <c r="AN11" s="10"/>
       <c r="AO11" s="30"/>
-      <c r="AU11" s="46"/>
-      <c r="AV11" s="46"/>
+      <c r="AU11" s="52"/>
+      <c r="AV11" s="52"/>
     </row>
     <row r="12" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A12">
@@ -1916,8 +1908,8 @@
       <c r="AM12" s="10"/>
       <c r="AN12" s="10"/>
       <c r="AO12" s="30"/>
-      <c r="AU12" s="46"/>
-      <c r="AV12" s="46"/>
+      <c r="AU12" s="52"/>
+      <c r="AV12" s="52"/>
     </row>
     <row r="13" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A13">
@@ -2002,8 +1994,8 @@
       <c r="AM13" s="10"/>
       <c r="AN13" s="10"/>
       <c r="AO13" s="30"/>
-      <c r="AU13" s="46"/>
-      <c r="AV13" s="46"/>
+      <c r="AU13" s="52"/>
+      <c r="AV13" s="52"/>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.2">
       <c r="A14">
@@ -2084,8 +2076,8 @@
       <c r="AM14" s="10"/>
       <c r="AN14" s="10"/>
       <c r="AO14" s="30"/>
-      <c r="AU14" s="46"/>
-      <c r="AV14" s="46"/>
+      <c r="AU14" s="52"/>
+      <c r="AV14" s="52"/>
     </row>
     <row r="15" spans="1:48" x14ac:dyDescent="0.2">
       <c r="D15" t="s">
@@ -2671,7 +2663,7 @@
     </row>
     <row r="27" spans="1:41" x14ac:dyDescent="0.2">
       <c r="B27" s="31" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D27" t="s">
         <v>52</v>
@@ -3441,7 +3433,7 @@
     </row>
     <row r="45" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="31" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D45" t="s">
         <v>52</v>
@@ -3951,7 +3943,7 @@
         <v>38</v>
       </c>
       <c r="D59" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E59">
         <v>1</v>
@@ -4033,7 +4025,7 @@
     </row>
     <row r="60" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A60" s="41" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B60" s="13"/>
       <c r="D60" t="s">
@@ -4127,7 +4119,7 @@
     </row>
     <row r="63" spans="1:40" x14ac:dyDescent="0.2">
       <c r="B63" s="31" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D63" t="s">
         <v>52</v>
@@ -4634,7 +4626,7 @@
         <v>12</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>13</v>
@@ -4646,7 +4638,7 @@
         <v>15</v>
       </c>
       <c r="R1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
@@ -4662,16 +4654,16 @@
         <v>a</v>
       </c>
       <c r="D2" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="G2" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="7"/>
@@ -4690,7 +4682,7 @@
         <v>16</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
@@ -4706,16 +4698,16 @@
         <v>b</v>
       </c>
       <c r="D3" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="G3" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H3" s="8"/>
       <c r="I3" s="7"/>
@@ -4747,16 +4739,16 @@
         <v>c</v>
       </c>
       <c r="D4" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H4" s="8"/>
       <c r="I4" s="7"/>
@@ -4787,16 +4779,16 @@
         <v>apple</v>
       </c>
       <c r="D5" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H5" s="8"/>
       <c r="I5" s="7"/>
@@ -4817,7 +4809,7 @@
         <v>18</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
@@ -4833,16 +4825,16 @@
         <v>e</v>
       </c>
       <c r="D6" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="G6" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H6" s="8"/>
       <c r="I6" s="7"/>
@@ -4859,10 +4851,10 @@
       <c r="O6" s="12"/>
       <c r="P6" s="11"/>
       <c r="Q6" s="11"/>
-      <c r="R6" s="55" t="s">
+      <c r="R6" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="S6" s="56"/>
+      <c r="S6" s="48"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="12">
@@ -4877,16 +4869,16 @@
         <v>f</v>
       </c>
       <c r="D7" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="7"/>
@@ -4917,16 +4909,16 @@
         <v>g</v>
       </c>
       <c r="D8" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="G8" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H8" s="8"/>
       <c r="I8" s="7"/>
@@ -4963,16 +4955,16 @@
         <v>qc</v>
       </c>
       <c r="D9" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H9" s="8"/>
       <c r="I9" s="7"/>
@@ -5015,16 +5007,16 @@
         <v>dm</v>
       </c>
       <c r="D10" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H10" s="8"/>
       <c r="I10" s="7"/>
@@ -5045,10 +5037,10 @@
       <c r="Q10" s="11">
         <v>1</v>
       </c>
-      <c r="R10" s="53" t="s">
+      <c r="R10" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="S10" s="54"/>
+      <c r="S10" s="46"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="12">
@@ -5063,16 +5055,16 @@
         <v>sysqc</v>
       </c>
       <c r="D11" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H11" s="8"/>
       <c r="I11" s="7"/>
@@ -5101,16 +5093,16 @@
         <v>bananas</v>
       </c>
       <c r="D12" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="G12" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H12" s="8"/>
       <c r="I12" s="7"/>
@@ -5129,7 +5121,7 @@
         <v>23</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
@@ -5145,16 +5137,16 @@
         <v>lib</v>
       </c>
       <c r="D13" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="G13" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H13" s="8"/>
       <c r="I13" s="7"/>
@@ -5164,17 +5156,15 @@
         <f>IF(LEN(User!AG13)=0,"",User!AG13)</f>
         <v/>
       </c>
-      <c r="M13" s="12">
-        <v>5</v>
-      </c>
+      <c r="M13" s="12"/>
       <c r="N13" s="12"/>
       <c r="O13" s="12"/>
       <c r="P13" s="11"/>
       <c r="Q13" s="11"/>
-      <c r="R13" s="53" t="s">
+      <c r="R13" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="S13" s="54"/>
+      <c r="S13" s="46"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="12">
@@ -5189,16 +5179,16 @@
         <v>qc2</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="G14" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="H14" s="8"/>
       <c r="I14" s="7"/>
@@ -5220,7 +5210,7 @@
         <v>1</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="S14" s="6" t="s">
         <v>98</v>
@@ -5256,7 +5246,7 @@
       <c r="P15" s="11"/>
       <c r="Q15" s="11"/>
       <c r="R15" s="43" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="S15" s="44"/>
     </row>
@@ -5290,7 +5280,7 @@
       <c r="P16" s="11"/>
       <c r="Q16" s="11"/>
       <c r="R16" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="S16" s="6"/>
     </row>
@@ -5323,10 +5313,10 @@
       <c r="O17" s="12"/>
       <c r="P17" s="11"/>
       <c r="Q17" s="11"/>
-      <c r="R17" s="58" t="s">
-        <v>100</v>
-      </c>
-      <c r="S17" s="57"/>
+      <c r="R17" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="S17" s="50"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="12">

</xml_diff>